<commit_message>
Verifica freelance IT: 6 SI_FREELANCE confermati, 4 spostati in Istituzioni, 2 non verificabili
</commit_message>
<xml_diff>
--- a/data/trainers_it/ErasmusDidactica_FORMATORI_IT_v1.xlsx
+++ b/data/trainers_it/ErasmusDidactica_FORMATORI_IT_v1.xlsx
@@ -478,25 +478,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ErasmusDidactica — FORMATORI_FREELANCE ITALIA (12 record)</t>
+          <t>ErasmusDidactica — FORMATORI_FREELANCE ITALIA (8 record)</t>
         </is>
       </c>
     </row>
@@ -551,6 +552,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICA_FREELANCE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -596,7 +602,12 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Presidente Impara Digitale. Google Certified Educator. Membro UNESCO. Collaboraz. FAO/WHO.</t>
+          <t>Presidente Impara Digitale. Google Certified Educator. Membro UNESCO. Collaboraz. FAO/WHO. VERIFICA: Presidente associazione Impara Digitale. Lavora con Samsung, Acer, Cisco, UNESCO, FAO. Chiaramente indipendente multi-cliente.</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
@@ -644,7 +655,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Formatore docenti trasformazione digitale. Bimed. Innovation Strategist.</t>
+          <t>Formatore docenti trasformazione digitale. Bimed. Innovation Strategist. VERIFICA: Co-founder KIIAI Innovation Lab. TEDx Speaker. Formatore per più scuole/enti. Profilo imprenditoriale.</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
@@ -692,34 +708,39 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Giornalista + formatore AI literacy. Consulente aziendale.</t>
+          <t>Giornalista + formatore AI literacy. Consulente aziendale. VERIFICA: Giornalista freelance dichiarato. Sito personale francescofacchini.it. Consulente AI per aziende+scuole. Membro AIFIA.</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>IT-T004</t>
+          <t>IT-T005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Vittorio Belloni</t>
+          <t>Alessandro Simoncini</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Didattica assistita tecnologie / STEAM / Magikering / Sostegno</t>
+          <t>AI per docenti / Percorsi educativi inclusivi con IA / Training Academy</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>STEAM</t>
+          <t>ICT/AI + Inclusione</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Gallarate (VA)</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -728,53 +749,62 @@
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alessandrosimoncini/</t>
+        </is>
+      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>https://www.imparadigitale.it/formatori/</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Docente sostegno ISIS Ponti. Creatore Magikering. Formatore Impara Digitale.</t>
+          <t>Corsi AI per insegnanti. Teoria+pratica. Percorsi inclusivi adattati. VERIFICA: Sito personale alessandrosimoncini.it. Lavora per Umana Forma + La Risorsa Umana + scuole. Multi-cliente = freelance.</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>IT-T005</t>
+          <t>IT-T008</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Alessandro Simoncini</t>
+          <t>Salvatore Paone</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>AI per docenti / Percorsi educativi inclusivi con IA / Training Academy</t>
+          <t>Creative &amp; Inclusive Learning / Robotica educativa / Visual programming / IA generativa</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ICT/AI + Inclusione</t>
+          <t>STEAM + Inclusione</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Milano</t>
+          <t>Firenze</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alessandrosimoncini/</t>
+          <t>https://www.linkedin.com/in/stranilivelli/</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -784,93 +814,103 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Corsi AI per insegnanti. Teoria+pratica. Percorsi inclusivi adattati.</t>
+          <t>Università di Firenze. Conferenze nazionali su apprendimento creativo e inclusivo. VERIFICA: Consulente IT, project manager, web designer dal 2006. Docente a contratto UniFI. Sito personale salvatorepaone.it. Multi-incarico = freelance.</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>IT-T008</t>
+          <t>IT-T012</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Salvatore Paone</t>
+          <t>Michele Maffucci</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Creative &amp; Inclusive Learning / Robotica educativa / Visual programming / IA generativa</t>
+          <t>STEAM / Robotica educativa / Arduino / Raspberry Pi / IA didattica / Coding</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>STEAM + Inclusione</t>
+          <t>STEAM + ICT/AI</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Firenze</t>
+          <t>Moncalieri (TO)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>FI</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/stranilivelli/</t>
-        </is>
-      </c>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>michele@maffucci.it</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>https://www.maffucci.it</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Università di Firenze. Conferenze nazionali su apprendimento creativo e inclusivo.</t>
+          <t>30+ anni esperienza. Formatore Tecnica della Scuola. Coordinatore lab PNRR. Referente CTS Torino. VERIFICA: Si definisce 'Maker, trainer, and freelance professional'. Sito personale maffucci.it. Email personale. Formatore Tecnica della Scuola. Multi-cliente.</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>SI_FREELANCE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>IT-T009</t>
+          <t>IT-T013</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Patrizia Mori</t>
+          <t>Giuseppe Fazzari</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Filosofia per bambini / Progetti educativi / Biblioteche scolastiche</t>
+          <t>Italiano L2 / Educazione interculturale / IA nella didattica / Tecnologie digitali</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Leadership + Lingue</t>
+          <t>Lingue + ICT/AI</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Firenze</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/patrizia-mori-9aba0534/</t>
+          <t>https://www.linkedin.com/in/giuseppe-fazzari/</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -880,45 +920,46 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Docente Facoltà Scienze Formazione Firenze. Formatrice pratica filosofica con bambini.</t>
+          <t>Insegnante e formatore italiano L2. Corsi con tecnologie digitali e approccio inclusivo. VERIFICA: Insegnante + formatore L2. Collabora con Centro Interculturale Torino. Non chiaro se ha P.IVA o solo incarichi.</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>NON_VERIFICABILE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>IT-T010</t>
+          <t>IT-T019</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Marianna Piccioli</t>
+          <t>Massimo Brizzi</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Inclusione scolastica / Modelli integrazione / Ricerca educativa Toscana</t>
+          <t>Formazione / Ottantaventi Formazione</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Inclusione</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Firenze</t>
-        </is>
-      </c>
+          <t>Leadership + SEL</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>MI</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/marianna-piccioli-72865192/</t>
+          <t>https://www.linkedin.com/in/massimo-brizzi/</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -928,201 +969,18 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Ricercatrice. Analisi PTOF Toscana su modelli inclusione scolastica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>IT-T012</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Michele Maffucci</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>STEAM / Robotica educativa / Arduino / Raspberry Pi / IA didattica / Coding</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>STEAM + ICT/AI</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Moncalieri (TO)</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>michele@maffucci.it</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.maffucci.it</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>30+ anni esperienza. Formatore Tecnica della Scuola. Coordinatore lab PNRR. Referente CTS Torino.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>IT-T013</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Giuseppe Fazzari</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Italiano L2 / Educazione interculturale / IA nella didattica / Tecnologie digitali</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Lingue + ICT/AI</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Torino</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/giuseppe-fazzari/</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Insegnante e formatore italiano L2. Corsi con tecnologie digitali e approccio inclusivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>IT-T014</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Massimiliano Ferrè</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Formazione docenti / VCO Formazione</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Piemonte</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/massimilianoferre/</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Formatore VCO Formazione. Area Piemonte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>IT-T019</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Massimo Brizzi</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Formazione / Ottantaventi Formazione</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Leadership + SEL</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>MI</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/massimo-brizzi/</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Formatore Ottantaventi Formazione. LinkedIn trovato.</t>
+          <t>Formatore Ottantaventi Formazione. LinkedIn trovato. VERIFICA: LinkedIn trovato. Ottantaventi Formazione. Non abbastanza info per verificare se freelance o dipendente.</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>NON_VERIFICABILE</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1134,25 +992,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ErasmusDidactica — ISTITUZIONI_PUBBLICHE ITALIA (7 record)</t>
+          <t>ErasmusDidactica — ISTITUZIONI_PUBBLICHE ITALIA (11 record)</t>
         </is>
       </c>
     </row>
@@ -1207,27 +1066,36 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>VERIFICA_FREELANCE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>IT-T006</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr"/>
+          <t>IT-T004</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Vittorio Belloni</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Formazione docenti digitale / KA1 accreditato Milano</t>
+          <t>Didattica assistita tecnologie / STEAM / Magikering / Sostegno</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>ICT/AI</t>
+          <t>STEAM</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Milano</t>
+          <t>Gallarate (VA)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1239,25 +1107,30 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://www.comune.milano.it/argomenti/scuola/progetti-scuola/erasmus-ka1</t>
+          <t>https://www.imparadigitale.it/formatori/</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Comune di Milano Erasmus+ KA1 accreditato 2021-2027.</t>
+          <t>Docente sostegno ISIS Ponti. Creatore Magikering. Formatore Impara Digitale. VERIFICA: Docente sostegno fisso ISIS Ponti Gallarate. Formatore solo per Impara Digitale. Nessuna evidenza attività freelance autonoma.</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>SOLO_DIPENDENTE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>IT-T007</t>
+          <t>IT-T006</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Didattica digitale / AI / Formazione docenti online</t>
+          <t>Formazione docenti digitale / KA1 accreditato Milano</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1275,238 +1148,444 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>formazione@tecnicadellascuola.it</t>
-        </is>
-      </c>
+      <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://corsi.tecnicadellascuola.it</t>
+          <t>https://www.comune.milano.it/argomenti/scuola/progetti-scuola/erasmus-ka1</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Tecnica della Scuola. Ente accreditato MIM. Tel 095 448780. Corsi SOFIA.</t>
-        </is>
-      </c>
+          <t>Comune di Milano Erasmus+ KA1 accreditato 2021-2027.</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>IT-T011</t>
+          <t>IT-T007</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Scienze della Formazione / Formazione insegnanti / Ricerca educativa</t>
+          <t>Didattica digitale / AI / Formazione docenti online</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Tutte</t>
+          <t>ICT/AI</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Firenze</t>
+          <t>Milano</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>FI</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>formazione@tecnicadellascuola.it</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.unifi.it</t>
+          <t>https://corsi.tecnicadellascuola.it</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Università di Firenze — Dipartimento Scienze Formazione. Potenziale partner accademico.</t>
-        </is>
-      </c>
+          <t>Tecnica della Scuola. Ente accreditato MIM. Tel 095 448780. Corsi SOFIA.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>IT-T015</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>IT-T009</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Patrizia Mori</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Formazione insegnanti / TFA / Inclusione scolastica / CIFIS</t>
+          <t>Filosofia per bambini / Progetti educativi / Biblioteche scolastiche</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Inclusione + Tutte</t>
+          <t>Leadership + Lingue</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Firenze</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>formazioneinsegnanti.piemonte@unito.it</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/patrizia-mori-9aba0534/</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.tfa-piemonte.unito.it</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Università di Torino — CIFIS. Esperto processi inclusione scolastica.</t>
+          <t>Docente Facoltà Scienze Formazione Firenze. Formatrice pratica filosofica con bambini. VERIFICA: Docente USR Firenze. Nessuna evidenza attività freelance autonoma. Formatrice interna Facoltà Scienze Formazione.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>SOLO_DIPENDENTE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>IT-T016</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr"/>
+          <t>IT-T010</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Marianna Piccioli</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Formazione professionale / Digitale / Inclusione</t>
+          <t>Inclusione scolastica / Modelli integrazione / Ricerca educativa Toscana</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>ICT/AI + Inclusione</t>
+          <t>Inclusione</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Mantova</t>
+          <t>Firenze</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/marianna-piccioli-72865192/</t>
+        </is>
+      </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.formazionemantova.it</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>For.Ma. — Azienda Speciale Formazione Mantova. Ente accreditato Regione Lombardia.</t>
+          <t>Ricercatrice. Analisi PTOF Toscana su modelli inclusione scolastica. VERIFICA: Ricercatrice Uni Roma Foro Italico (strutturata). Ex-assegnista UniFI. Profilo accademico puro.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>SOLO_DIPENDENTE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>IT-T017</t>
+          <t>IT-T011</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Digitale scuola / PNRR / Coding / Robotica / IA</t>
+          <t>Scienze della Formazione / Formazione insegnanti / Ricerca educativa</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>ICT/AI + STEAM</t>
+          <t>Tutte</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Vigevano (PV) — area Lombardia</t>
+          <t>Firenze</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>MN</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>digitalschoolacademy@liceocairoli.edu.it</t>
-        </is>
-      </c>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>https://www.digitalschoolacademy.it</t>
+          <t>https://www.unifi.it</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Digital School Academy. Polo formativo nazionale PNRR. Tel +39 0381 84215.</t>
-        </is>
-      </c>
+          <t>Università di Firenze — Dipartimento Scienze Formazione. Potenziale partner accademico.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>IT-T014</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Massimiliano Ferrè</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Formazione docenti / VCO Formazione</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Leadership</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Piemonte</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/massimilianoferre/</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Formatore VCO Formazione. Area Piemonte. VERIFICA: Dipendente VCO Formazione (ente accreditato Regione Piemonte). Area Innovation. Non freelance.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>SOLO_DIPENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>IT-T015</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Formazione insegnanti / TFA / Inclusione scolastica / CIFIS</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Inclusione + Tutte</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Torino</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>formazioneinsegnanti.piemonte@unito.it</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tfa-piemonte.unito.it</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Università di Torino — CIFIS. Esperto processi inclusione scolastica.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>IT-T016</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Formazione professionale / Digitale / Inclusione</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ICT/AI + Inclusione</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Mantova</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.formazionemantova.it</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>For.Ma. — Azienda Speciale Formazione Mantova. Ente accreditato Regione Lombardia.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>IT-T017</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Digitale scuola / PNRR / Coding / Robotica / IA</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>ICT/AI + STEAM</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Vigevano (PV) — area Lombardia</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>digitalschoolacademy@liceocairoli.edu.it</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.digitalschoolacademy.it</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Digital School Academy. Polo formativo nazionale PNRR. Tel +39 0381 84215.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>IT-T018</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Équipe Formativa Territoriale Lombardia / Digitale scuole</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>ICT/AI</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Milano (tutta Lombardia)</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>drlo.equipe@istruzione.it</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>https://www.eftlombardia.it</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>27 docenti. Coord. Dott.ssa Nicoletta Falcone. Helpdesk per scuole.</t>
         </is>
       </c>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1518,19 +1597,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1591,6 +1671,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>VERIFICA_FREELANCE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1631,6 +1716,7 @@
           <t>Erasmus Learning Academy. OID E10221762. CONCORRENTE diretto.</t>
         </is>
       </c>
+      <c r="K3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -1667,6 +1753,7 @@
           <t>Europass Teacher Academy. CONCORRENTE principale. Sede Firenze.</t>
         </is>
       </c>
+      <c r="K4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1703,10 +1790,11 @@
           <t>EGInA srl. Provider KA1. CONCORRENTE.</t>
         </is>
       </c>
+      <c r="K5" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>